<commit_message>
Fix settings form save state desync and update UI glass styling
</commit_message>
<xml_diff>
--- a/test_questions.xlsx
+++ b/test_questions.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10713"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bacond\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1bb832f76a8146a2/Documents/BU_SE/QuizYou/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_04D6B35CB6314872E4BFB9261D1F5E282AD287C2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -77,7 +78,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -388,11 +389,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -415,7 +416,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -438,7 +439,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -461,7 +462,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -472,7 +473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>15</v>
       </c>

</xml_diff>